<commit_message>
Hogar de Refugio: sustento normativo cotejado con la R.V.M. 208-2019-MINEDU
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/MATRIZ_SUSTENTO_NORMATIVO_PROGRAMA_ARQUITECTONICO_HOGAR_REFUGIO.xlsx
+++ b/entregables/MATRIZ_SUSTENTO_NORMATIVO_PROGRAMA_ARQUITECTONICO_HOGAR_REFUGIO.xlsx
@@ -797,7 +797,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 2.4</t>
+          <t>R.V.M. 208-2019 cuadro 40; lineamientos 2.4</t>
         </is>
       </c>
       <c r="G9" s="8" t="n"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="O9" s="6" t="inlineStr">
         <is>
-          <t>Con 1 persona a 3.00 m² por persona (R.V.M. 208-2019), el área mínima es de 3.00 m², y el ambiente tiene 10.00 m². Caseta de vigilancia en el acceso principal, con servicio higiénico para el personal de guardia, comunicación interna y control de los accesos (lineamientos 2.4 y 2.6; R.V.M. 104-2019 num. 13.3.2).</t>
+          <t>Con 1 persona a 3.00 m² por persona (R.V.M. 208-2019 cuadro 40), el área mínima es de 3.00 m², y el ambiente tiene 10.00 m². Caseta de control junto al ingreso principal con servicio higiénico de 01 lavadero y 01 inodoro para el personal de guardia (R.V.M. 208-2019 num. 12.3.3), comunicación interna y control de los accesos (lineamientos 2.4 y 2.6).</t>
         </is>
       </c>
     </row>
@@ -1526,10 +1526,12 @@
       <c r="E24" s="8" t="n"/>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 num. 13.3.5</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="n"/>
+          <t>R.V.M. 208-2019 num. 12.3.6 y cuadro 40</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>1.5</v>
+      </c>
       <c r="H24" s="8">
         <f>IF(AND(ISNUMBER(D24),ISNUMBER(E24)),D24*E24,IF(ISNUMBER(G24),G24,"—"))</f>
         <v/>
@@ -1552,7 +1554,7 @@
       </c>
       <c r="O24" s="6" t="inlineStr">
         <is>
-          <t>Guardado de implementos de limpieza, con lavadero y sumidero (R.V.M. 104-2019 num. 13.3.5).</t>
+          <t>El área mínima es de 1.50 m² y el ambiente tiene 4.80 m². Guardado de implementos de limpieza con lavadero (R.V.M. 208-2019 num. 12.3.6; R.V.M. 104-2019 num. 13.3.5).</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1778,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1">
+    <row r="29" ht="48" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Zona administrativa</t>
@@ -1828,11 +1830,11 @@
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>Con 3 personas a 10.00 m² por persona (A.090 art. 11), el área mínima es de 30.00 m², y el ambiente tiene 30.00 m². Supera la superficie sugerida por los lineamientos (9.00 a 14.00 m²). Mayor que el tópico de la R.V.M. 104-2019 (7.00 m², cuadro 22).</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="36" customHeight="1">
+          <t>Con 3 personas a 10.00 m² por persona (A.090 art. 11), el área mínima es de 30.00 m², y el ambiente tiene 30.00 m². Supera la superficie sugerida por los lineamientos (9.00 a 14.00 m²). Mayor que el tópico de la R.V.M. 104-2019 (7.00 m², cuadro 22) y que el de la R.V.M. 208-2019 (9.00 m² con personal fijo, cuadro 31).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Zona administrativa</t>
@@ -1854,7 +1856,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 2.4</t>
+          <t>R.V.M. 208-2019 num. 12.3.3 y cuadro 40; lineamientos 2.4</t>
         </is>
       </c>
       <c r="G30" s="8" t="n"/>
@@ -1880,7 +1882,7 @@
       </c>
       <c r="O30" s="6" t="inlineStr">
         <is>
-          <t>Con 4 personas a 3.00 m² por persona (R.V.M. 208-2019), el área mínima es de 12.00 m², y el ambiente tiene 15.00 m². Monitoreo del circuito cerrado de accesos, perímetro y áreas comunes (lineamientos 2.4 y 2.5).</t>
+          <t>Con 4 personas a 3.00 m² por persona (R.V.M. 208-2019 cuadro 40), el área mínima es de 12.00 m², y el ambiente tiene 15.00 m². Monitoreo del circuito cerrado de vigilancia (R.V.M. 208-2019 num. 12.3.3 c) de accesos, perímetro y áreas comunes (lineamientos 2.4 y 2.5), con el índice de la caseta de control.</t>
         </is>
       </c>
     </row>
@@ -1954,7 +1956,7 @@
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 cuadro 21</t>
+          <t>R.V.M. 208-2019 cuadro 29</t>
         </is>
       </c>
       <c r="G32" s="8" t="n">
@@ -1982,7 +1984,7 @@
       </c>
       <c r="O32" s="6" t="inlineStr">
         <is>
-          <t>El área mínima es de 6.00 m² y el ambiente tiene 12.00 m². R.V.M. 104-2019: archivo de 6.00 m², contiguo a las oficinas.</t>
+          <t>El área mínima es de 6.00 m² y el ambiente tiene 12.00 m². Archivo de 6.00 m², contiguo o integrado al área de oficinas (R.V.M. 208-2019 cuadro 29; R.V.M. 104-2019 cuadro 21).</t>
         </is>
       </c>
     </row>
@@ -2006,11 +2008,11 @@
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 num. 13.3.1</t>
+          <t>R.V.M. 208-2019 cuadro 29</t>
         </is>
       </c>
       <c r="G33" s="8" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H33" s="8">
         <f>IF(AND(ISNUMBER(D33),ISNUMBER(E33)),D33*E33,IF(ISNUMBER(G33),G33,"—"))</f>
@@ -2034,7 +2036,7 @@
       </c>
       <c r="O33" s="6" t="inlineStr">
         <is>
-          <t>El área mínima es de 10.00 m² y el ambiente tiene 15.00 m². R.V.M. 104-2019: almacén o depósito no menor de 10.00 m².</t>
+          <t>El área mínima es de 4.00 m² y el ambiente tiene 15.00 m². Depósito de materiales de oficina de 4.00 m², contiguo o integrado al área de oficinas (R.V.M. 208-2019 cuadro 29).</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2061,7 @@
       <c r="N34" s="5" t="n"/>
       <c r="O34" s="5" t="n"/>
     </row>
-    <row r="35" ht="36" customHeight="1">
+    <row r="35" ht="48" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Zona de ambientes especializados</t>
@@ -2081,7 +2083,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>A.040 art. 13</t>
+          <t>R.V.M. 208-2019 cuadro 20; A.040 art. 13</t>
         </is>
       </c>
       <c r="G35" s="8" t="n"/>
@@ -2109,11 +2111,11 @@
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>Con 20 personas a 3.00 m² por persona (A.040 art. 13), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="36" customHeight="1">
+          <t>Con 20 personas a 3.00 m² por persona (R.V.M. 208-2019 cuadro 20), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7); el índice coincide con el de talleres de la A.040 (3.0 m²/persona).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Zona de ambientes especializados</t>
@@ -2135,7 +2137,7 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>A.040 art. 13</t>
+          <t>R.V.M. 208-2019 cuadro 20; A.040 art. 13</t>
         </is>
       </c>
       <c r="G36" s="8" t="n"/>
@@ -2163,11 +2165,11 @@
       </c>
       <c r="O36" s="6" t="inlineStr">
         <is>
-          <t>Con 20 personas a 3.00 m² por persona (A.040 art. 13), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7).</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="36" customHeight="1">
+          <t>Con 20 personas a 3.00 m² por persona (R.V.M. 208-2019 cuadro 20), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7); el índice coincide con el de talleres de la A.040 (3.0 m²/persona).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Zona de ambientes especializados</t>
@@ -2189,7 +2191,7 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>A.040 art. 13</t>
+          <t>R.V.M. 208-2019 cuadro 20; A.040 art. 13</t>
         </is>
       </c>
       <c r="G37" s="8" t="n"/>
@@ -2217,7 +2219,7 @@
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
-          <t>Con 20 personas a 3.00 m² por persona (A.040 art. 13), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7).</t>
+          <t>Con 20 personas a 3.00 m² por persona (R.V.M. 208-2019 cuadro 20), el área mínima es de 60.00 m², y el ambiente tiene 60.00 m². Supera la superficie sugerida por los lineamientos (45.00 m²). Taller productivo para la autonomía económica de las usuarias (lineamientos 3.7); el índice coincide con el de talleres de la A.040 (3.0 m²/persona).</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2335,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="36" customHeight="1">
+    <row r="40" ht="48" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Zona de ambientes especializados</t>
@@ -2351,11 +2353,11 @@
         <v>15</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 cuadro 16</t>
+          <t>R.V.M. 208-2019 cuadro 12</t>
         </is>
       </c>
       <c r="G40" s="8" t="n"/>
@@ -2385,7 +2387,7 @@
       </c>
       <c r="O40" s="6" t="inlineStr">
         <is>
-          <t>Con 15 personas a 2.40 m² por persona (R.V.M. 104-2019 cuadro 16), el área mínima es de 36.00 m², y el ambiente tiene 39.00 m². Supera la superficie sugerida por los lineamientos (16.00 a 21.00 m²). Continuidad educativa de niñas y niños (lineamientos 3.5).</t>
+          <t>Con 15 personas a 2.00 m² por persona (R.V.M. 208-2019 cuadro 12), el área mínima es de 30.00 m², y el ambiente tiene 39.00 m². Supera la superficie sugerida por los lineamientos (16.00 a 21.00 m²). Continuidad educativa de niñas y niños (lineamientos 3.5). Cumple también el aula de inicial de la R.V.M. 104-2019 (cuadro 16, 2.40 m²: 36.00 m²).</t>
         </is>
       </c>
     </row>
@@ -3284,15 +3286,15 @@
       <c r="D59" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="E59" s="8" t="n">
-        <v>6</v>
-      </c>
+      <c r="E59" s="8" t="n"/>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 3.2</t>
-        </is>
-      </c>
-      <c r="G59" s="8" t="n"/>
+          <t>Lineamientos 3.2; R.V.M. 208-2019 anexo 4</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="n">
+        <v>32</v>
+      </c>
       <c r="H59" s="8">
         <f>IF(AND(ISNUMBER(D59),ISNUMBER(E59)),D59*E59,IF(ISNUMBER(G59),G59,"—"))</f>
         <v/>
@@ -3315,11 +3317,11 @@
       </c>
       <c r="O59" s="6" t="inlineStr">
         <is>
-          <t>Con 6 personas a 6.00 m² por persona (R.V.M. 208-2019), el área mínima es de 36.00 m², y el ambiente tiene 36.00 m². Supera los 0.40 m² por comensal de los lineamientos (80 x 0.40 = 32.00 m²); acceso restringido a niñas y niños.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="36" customHeight="1">
+          <t>El área mínima es de 32.00 m² y el ambiente tiene 36.00 m². La R.V.M. 208-2019 remite el dimensionamiento de la cocina a la normativa que la regula (anexo 4, cocina escolar); con 0.40 m² por comensal (lineamientos 3.2) los 80 comensales requieren 32.00 m². Acceso restringido a niñas y niños.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="24" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Zona de servicios complementarios</t>
@@ -3336,12 +3338,10 @@
       <c r="D60" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E60" s="8" t="n">
-        <v>6</v>
-      </c>
+      <c r="E60" s="8" t="n"/>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 3.2</t>
+          <t>Lineamientos 3.2; R.V.M. 208-2019 anexo 4</t>
         </is>
       </c>
       <c r="G60" s="8" t="n"/>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="O60" s="6" t="inlineStr">
         <is>
-          <t>Con 1 persona a 6.00 m² por persona (R.V.M. 208-2019), el área mínima es de 6.00 m², y el ambiente tiene 6.00 m². Con la alacena (9.00 m²) suma 15.00 m² de almacenamiento de alimentos, por encima de la superficie sugerida para la despensa (9/12 m², lineamientos 3.2).</t>
+          <t>Con la alacena (9.00 m²) suma 15.00 m² de almacenamiento de alimentos, por encima de la superficie sugerida para la despensa (9/12 m², lineamientos 3.2).</t>
         </is>
       </c>
     </row>
@@ -3388,12 +3388,10 @@
       <c r="D61" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E61" s="8" t="n">
-        <v>6</v>
-      </c>
+      <c r="E61" s="8" t="n"/>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019</t>
+          <t>Lineamientos 3.2; R.V.M. 208-2019 anexo 4</t>
         </is>
       </c>
       <c r="G61" s="8" t="n"/>
@@ -3419,11 +3417,11 @@
       </c>
       <c r="O61" s="6" t="inlineStr">
         <is>
-          <t>Con 1 persona a 6.00 m² por persona (R.V.M. 208-2019), el área mínima es de 6.00 m², y el ambiente tiene 9.00 m². Complementa la despensa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="36" customHeight="1">
+          <t>Complementa la despensa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="48" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
           <t>Zona de servicios complementarios</t>
@@ -3445,7 +3443,7 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>A.040 art. 13</t>
+          <t>R.V.M. 208-2019 cuadro 22; A.040 art. 13</t>
         </is>
       </c>
       <c r="G62" s="8" t="n"/>
@@ -3471,11 +3469,11 @@
       </c>
       <c r="O62" s="6" t="inlineStr">
         <is>
-          <t>Con 80 personas a 1.00 m² por persona (A.040 art. 13), el área mínima es de 80.00 m², y el ambiente tiene 240.00 m². Con 1.00 m² por residente (lineamientos 3.2), sus 240.00 m² permiten atender a la totalidad de las residentes en un solo turno.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="36" customHeight="1">
+          <t>Con 80 personas a 1.00 m² por persona (R.V.M. 208-2019 cuadro 22), el área mínima es de 80.00 m², y el ambiente tiene 240.00 m². La R.V.M. 208-2019 (num. 11.4.1 e) admite las actividades de alimentación en la SUM. Con 1.00 m² por residente (lineamientos 3.2), sus 240.00 m² permiten atender a la totalidad de las residentes en un solo turno, por debajo del máximo de 300 m² de la norma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="48" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
           <t>Zona de servicios complementarios</t>
@@ -3497,7 +3495,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 3.4</t>
+          <t>R.V.M. 208-2019 num. 12.2.1 i; lineamientos 3.4</t>
         </is>
       </c>
       <c r="G63" s="8" t="n"/>
@@ -3523,7 +3521,7 @@
       </c>
       <c r="O63" s="6" t="inlineStr">
         <is>
-          <t>Con 12 personas a 3.00 m² por persona (R.V.M. 208-2019), el área mínima es de 36.00 m², y el ambiente tiene 36.00 m². Lavado, secado y planchado con tendido al aire libre y cubierto (lineamientos 3.4).</t>
+          <t>Con 12 personas a 3.00 m² por persona (R.V.M. 208-2019 num. 12.2.1 i), el área mínima es de 36.00 m², y el ambiente tiene 36.00 m². El índice se aplica a la mitad de las usuarias del espacio y el área puede reducirse con máquinas lavadoras (R.V.M. 208-2019 num. 12.2.1 i). Lavado, secado y planchado con tendido al aire libre y cubierto (lineamientos 3.4).</t>
         </is>
       </c>
     </row>
@@ -3593,7 +3591,7 @@
       <c r="E65" s="8" t="n"/>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019</t>
+          <t>R.V.M. 208-2019 num. 11.6.3</t>
         </is>
       </c>
       <c r="G65" s="8" t="n"/>
@@ -3619,7 +3617,7 @@
       </c>
       <c r="O65" s="6" t="inlineStr">
         <is>
-          <t>Área exterior de reunión y recreación (lineamientos 3.9).</t>
+          <t>Espacio exterior de socialización y recreación (R.V.M. 208-2019 num. 11.6.3; lineamientos 3.9).</t>
         </is>
       </c>
     </row>
@@ -3741,10 +3739,12 @@
       <c r="E68" s="8" t="n"/>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>Lineamientos 3.9</t>
-        </is>
-      </c>
-      <c r="G68" s="8" t="n"/>
+          <t>R.V.M. 208-2019 cuadro 23</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="n">
+        <v>800</v>
+      </c>
       <c r="H68" s="8">
         <f>IF(AND(ISNUMBER(D68),ISNUMBER(E68)),D68*E68,IF(ISNUMBER(G68),G68,"—"))</f>
         <v/>
@@ -3756,9 +3756,7 @@
         <f>IF(AND(ISNUMBER(H68),ISNUMBER(I68)),IF(I68&gt;=H68-0.001,"CUMPLE","NO CUMPLE"),"CONFORME")</f>
         <v/>
       </c>
-      <c r="K68" s="8" t="n">
-        <v>420</v>
-      </c>
+      <c r="K68" s="8" t="n"/>
       <c r="L68" s="8" t="n"/>
       <c r="M68" s="7">
         <f>IF(AND(ISNUMBER(K68),ISNUMBER(I68)),IF(AND(ISNUMBER(L68),I68&lt;=L68),"EN RANGO","SUPERA"),"—")</f>
@@ -3769,7 +3767,7 @@
       </c>
       <c r="O68" s="6" t="inlineStr">
         <is>
-          <t>Supera la superficie sugerida por los lineamientos (420.00 m²). Permite canchas de básquet (15 x 28 m) y voleibol (9 x 18 m) (lineamientos 3.9).</t>
+          <t>El área mínima es de 800.00 m² y el ambiente tiene 809.00 m². Losa multiuso tipo II de la R.V.M. 208-2019 (20 x 40 m, 800 m²), que permite fútbol sala, básquet y vóley (lineamientos 3.9).</t>
         </is>
       </c>
     </row>
@@ -3839,10 +3837,12 @@
       <c r="E70" s="8" t="n"/>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019</t>
-        </is>
-      </c>
-      <c r="G70" s="8" t="n"/>
+          <t>R.V.M. 208-2019 num. 11.5.8 y cuadro 40</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="n">
+        <v>16</v>
+      </c>
       <c r="H70" s="8">
         <f>IF(AND(ISNUMBER(D70),ISNUMBER(E70)),D70*E70,IF(ISNUMBER(G70),G70,"—"))</f>
         <v/>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="O70" s="6" t="inlineStr">
         <is>
-          <t>Guardado de implementos deportivos.</t>
+          <t>El área mínima es de 16.00 m² y el ambiente tiene 20.50 m². Depósito de implementos deportivos del tipo I de la R.V.M. 208-2019 (16.00 m²), ventilado y con estantes.</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="24" customHeight="1">
+    <row r="73" ht="36" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
           <t>Zona de servicios generales</t>
@@ -3960,7 +3960,7 @@
       <c r="E73" s="8" t="n"/>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 num. 13.3.1</t>
+          <t>R.V.M. 208-2019 num. 12.3.1</t>
         </is>
       </c>
       <c r="G73" s="8" t="n">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="O73" s="6" t="inlineStr">
         <is>
-          <t>El área mínima es de 10.00 m² y el ambiente tiene 17.60 m². R.V.M. 104-2019: almacén general no menor de 10.00 m²; productos de limpieza bajo llave (lineamientos 2.5).</t>
+          <t>El área mínima es de 10.00 m² y el ambiente tiene 17.60 m². Almacén general no menor de 10.00 m² (R.V.M. 208-2019 num. 12.3.1; R.V.M. 104-2019 num. 13.3.1); productos de limpieza bajo llave (lineamientos 2.5).</t>
         </is>
       </c>
     </row>
@@ -4009,12 +4009,10 @@
       <c r="D74" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="E74" s="8" t="n">
-        <v>3</v>
-      </c>
+      <c r="E74" s="8" t="n"/>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019</t>
+          <t>R.V.M. 208-2019 num. 12.3.2</t>
         </is>
       </c>
       <c r="G74" s="8" t="n"/>
@@ -4040,7 +4038,7 @@
       </c>
       <c r="O74" s="6" t="inlineStr">
         <is>
-          <t>Con 4 personas a 3.00 m² por persona (R.V.M. 208-2019), el área mínima es de 12.00 m², y el ambiente tiene 15.00 m². Mantenimiento del local.</t>
+          <t>Taller de mantenimiento del local (R.V.M. 208-2019 num. 12.3.2), dimensionado para el personal y el equipo de mantenimiento del hogar.</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4062,7 @@
       <c r="E75" s="8" t="n"/>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>A.080 art. 23; R.V.M. 104-2019 num. 13.3.4</t>
+          <t>A.080 art. 23; R.V.M. 208-2019 num. 12.3.5</t>
         </is>
       </c>
       <c r="G75" s="8" t="n">
@@ -4116,7 +4114,7 @@
       <c r="E76" s="8" t="n"/>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>EM.010; R.V.M. 104-2019 num. 13.3.6</t>
+          <t>EM.010; R.V.M. 208-2019 num. 12.3.7</t>
         </is>
       </c>
       <c r="G76" s="8" t="n"/>
@@ -4142,7 +4140,7 @@
       </c>
       <c r="O76" s="6" t="inlineStr">
         <is>
-          <t>Fuera del alcance de niñas y niños (R.V.M. 104-2019 num. 13.3.6).</t>
+          <t>Sobre el nivel del suelo, ventilado y de acceso restringido; área según la carga instalada (R.V.M. 208-2019 num. 12.3.7), fuera del alcance de niñas y niños.</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4164,7 @@
       <c r="E77" s="8" t="n"/>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 104-2019 num. 13.3.3</t>
+          <t>R.V.M. 208-2019 num. 12.3.4</t>
         </is>
       </c>
       <c r="G77" s="8" t="n"/>
@@ -4192,7 +4190,7 @@
       </c>
       <c r="O77" s="6" t="inlineStr">
         <is>
-          <t>Acceso solo del personal autorizado.</t>
+          <t>Sobre el nivel del suelo, ventilado y de acceso solo del personal de mantenimiento (R.V.M. 208-2019 num. 12.3.4).</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4216,7 @@
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>R.V.M. 208-2019; lineamientos 2.4</t>
+          <t>R.V.M. 208-2019 cuadro 40; lineamientos 2.4</t>
         </is>
       </c>
       <c r="G78" s="8" t="n"/>
@@ -4244,7 +4242,7 @@
       </c>
       <c r="O78" s="6" t="inlineStr">
         <is>
-          <t>Con 1 persona a 3.00 m² por persona (R.V.M. 208-2019), el área mínima es de 3.00 m², y el ambiente tiene 10.00 m². Caseta de control de los accesos de servicio (lineamientos 2.4).</t>
+          <t>Con 1 persona a 3.00 m² por persona (R.V.M. 208-2019 cuadro 40), el área mínima es de 3.00 m², y el ambiente tiene 10.00 m². Caseta de control de los accesos de servicio (lineamientos 2.4).</t>
         </is>
       </c>
     </row>
@@ -4834,7 +4832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5197,6 +5195,106 @@
       </c>
       <c r="D20" s="12" t="n">
         <v>1.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>R208aula</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>R.V.M. 208-2019 cuadro 12</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Aula: capacidad 30 estudiantes, I.O. 2.00 m², área 60.00 m².</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>R208tal</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>R.V.M. 208-2019 cuadro 20</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Taller creativo / taller de arte: capacidad 30 estudiantes, I.O. 3.00 m², área 90.00 m² (incluye depósito de aprox. 15 % del área).</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>R208sum</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>R.V.M. 208-2019 cuadro 22</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Sala de usos múltiples: I.O. 1.00 m²; con 5 o más secciones el área no debe ser mayor a 300 m².</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>R208lav</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>R.V.M. 208-2019 num. 12.2.1 i</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Lavandería: I.O. de 3.00 m² por 1/2 de la cantidad total de usuarios que hacen uso de este espacio; puede reducirse si se cuenta con máquinas lavadoras.</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>R208cas</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>R.V.M. 208-2019 cuadro 40</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Vigilancia / caseta de control: área 3.00 m², I.O. 3.00 m², 01 usuario.</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -5466,12 +5564,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Programación arquitectónica</t>
+          <t>Arts. 11 y 12; cuadros 12, 20, 22, 23, 29 y 40</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Índices citados en la programación para cocina, comedor/SUM, lavandería, patios, losa y servicios generales.</t>
+          <t>Módulo de enseñanza, talleres, comedor/SUM, losa multiuso, archivo, depósitos, caseta de control, lavandería, almacenes y servicios generales.</t>
         </is>
       </c>
     </row>

</xml_diff>